<commit_message>
v5 upload working ribo seq metadata
</commit_message>
<xml_diff>
--- a/test-datasets/Testtemplate.xlsx
+++ b/test-datasets/Testtemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mikej10\advbfx\flowAPIscripts\test-datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FD4EFE6-5EAF-4731-8561-9F2D474F76BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5650B363-DEB2-49C7-B4D1-606794B0F40A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2295" yWindow="2295" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -245,52 +245,52 @@
     <t>Separation Method</t>
   </si>
   <si>
+    <t>Sucrose gradient</t>
+  </si>
+  <si>
+    <t>E130_6_ASO_3</t>
+  </si>
+  <si>
+    <t>riboseq, no sucrose gradient</t>
+  </si>
+  <si>
+    <t>Size selection</t>
+  </si>
+  <si>
+    <t>Ribosome stabilization method</t>
+  </si>
+  <si>
+    <t>brain</t>
+  </si>
+  <si>
+    <t>whOrg1_B12_hOrg33d_c2</t>
+  </si>
+  <si>
+    <t>SRR2967100.fastq.gz</t>
+  </si>
+  <si>
+    <t>scRNA</t>
+  </si>
+  <si>
+    <t>F344/Stm frontal cortex sample</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Strandedness (Required)</t>
+  </si>
+  <si>
+    <t>E130_trimmed.fastq.gz</t>
+  </si>
+  <si>
+    <t>PHO92_A_1.fastq.gz</t>
+  </si>
+  <si>
+    <t>ERR11899255_trim.fastq.gz</t>
+  </si>
+  <si>
     <t>broad selection (25-35 nt)</t>
-  </si>
-  <si>
-    <t>Sucrose gradient</t>
-  </si>
-  <si>
-    <t>E130_6_ASO_3</t>
-  </si>
-  <si>
-    <t>riboseq, no sucrose gradient</t>
-  </si>
-  <si>
-    <t>Size selection</t>
-  </si>
-  <si>
-    <t>Ribosome stabilization method</t>
-  </si>
-  <si>
-    <t>brain</t>
-  </si>
-  <si>
-    <t>whOrg1_B12_hOrg33d_c2</t>
-  </si>
-  <si>
-    <t>SRR2967100.fastq.gz</t>
-  </si>
-  <si>
-    <t>scRNA</t>
-  </si>
-  <si>
-    <t>F344/Stm frontal cortex sample</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Strandedness (Required)</t>
-  </si>
-  <si>
-    <t>E130_trimmed.fastq.gz</t>
-  </si>
-  <si>
-    <t>PHO92_A_1.fastq.gz</t>
-  </si>
-  <si>
-    <t>ERR11899255_trim.fastq.gz</t>
   </si>
 </sst>
 </file>
@@ -792,7 +792,7 @@
         <v>23</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Z1" s="1" t="s">
         <v>24</v>
@@ -801,7 +801,7 @@
         <v>25</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AC1" s="2" t="s">
         <v>64</v>
@@ -810,18 +810,18 @@
         <v>65</v>
       </c>
       <c r="AE1" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="AF1" s="2" t="s">
         <v>69</v>
       </c>
       <c r="AG1" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B2" t="s">
         <v>47</v>
@@ -904,7 +904,7 @@
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B3" t="s">
         <v>57</v>
@@ -987,10 +987,10 @@
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
         <v>46</v>
@@ -1005,7 +1005,7 @@
         <v>53</v>
       </c>
       <c r="H4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I4" t="s">
         <v>50</v>
@@ -1068,15 +1068,15 @@
         <v>68</v>
       </c>
       <c r="AF4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AG4" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
         <v>46</v>
@@ -1218,10 +1218,10 @@
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C7" t="s">
         <v>46</v>
@@ -1236,7 +1236,7 @@
         <v>53</v>
       </c>
       <c r="H7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I7" t="s">
         <v>50</v>
@@ -1287,7 +1287,7 @@
         <v>48</v>
       </c>
       <c r="Y7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Z7" t="s">
         <v>28</v>

</xml_diff>